<commit_message>
updated design excel sheet
</commit_message>
<xml_diff>
--- a/Design_Formulas.xlsx
+++ b/Design_Formulas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Drones\ORGOfly-CAD-model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A1097411\Documents\GitHub\ORGOfly-CAD-model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4497F99-A021-408B-A773-BB85CF071D31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E96A58A-9758-43AD-A053-8AE727531577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{9597FAC8-E3BA-4239-B29C-D9DA52C8E4BB}"/>
+    <workbookView xWindow="30435" yWindow="3150" windowWidth="21600" windowHeight="11235" activeTab="2" xr2:uid="{9597FAC8-E3BA-4239-B29C-D9DA52C8E4BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Constants" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="63">
   <si>
     <t>kg</t>
   </si>
@@ -95,9 +95,6 @@
   </si>
   <si>
     <t>Assumed average viscosity of the air at standard conditions between 10 and 15deg and SOF atmospheric pressure</t>
-  </si>
-  <si>
-    <t>m^2/s</t>
   </si>
   <si>
     <t>m</t>
@@ -164,9 +161,6 @@
     <t>aspect ratio</t>
   </si>
   <si>
-    <t>m^2</t>
-  </si>
-  <si>
     <t>mean wing chord</t>
   </si>
   <si>
@@ -220,21 +214,6 @@
     <t>moment arm to the VT from wing AC to tail AC</t>
   </si>
   <si>
-    <r>
-      <t>S</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>VT</t>
-    </r>
-  </si>
-  <si>
     <t>area of the vertical tail</t>
   </si>
   <si>
@@ -354,6 +333,67 @@
   <si>
     <t>V-tail surface area</t>
   </si>
+  <si>
+    <r>
+      <t>m</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>VT</t>
+    </r>
+  </si>
+  <si>
+    <t>Final Results</t>
+  </si>
+  <si>
+    <r>
+      <t>m</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/s</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -363,7 +403,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -407,6 +447,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <vertAlign val="superscript"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <vertAlign val="subscript"/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -440,7 +496,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -583,11 +639,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -662,31 +744,25 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -703,6 +779,18 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1552,7 +1640,7 @@
       <xdr:col>14</xdr:col>
       <xdr:colOff>572637</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>30465</xdr:rowOff>
+      <xdr:rowOff>18559</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2152,7 +2240,7 @@
       <xdr:col>22</xdr:col>
       <xdr:colOff>441959</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>148590</xdr:rowOff>
+      <xdr:rowOff>136684</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3067,8 +3155,8 @@
       <xdr:rowOff>185736</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="2324100" cy="177228"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="TextBox 1">
@@ -3110,6 +3198,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -3302,7 +3391,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="TextBox 1">
@@ -3759,34 +3848,34 @@
     </row>
     <row r="7" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="43" t="s">
+      <c r="B8" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="44" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="44" t="s">
+      <c r="C8" s="42" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="44" t="s">
+      <c r="E8" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="44" t="s">
+      <c r="F8" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="44" t="s">
+      <c r="G8" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="45" t="s">
+      <c r="H8" s="43" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="B9" s="49" t="s">
+      <c r="B9" s="47" t="s">
         <v>1</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D9" s="4">
         <v>15</v>
@@ -3815,7 +3904,7 @@
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="4">
@@ -3830,10 +3919,10 @@
     </row>
     <row r="12" spans="2:8" ht="45" x14ac:dyDescent="0.25">
       <c r="B12" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D12" s="4">
         <v>1.4</v>
@@ -3841,13 +3930,13 @@
       <c r="E12" s="4"/>
       <c r="F12" s="10"/>
       <c r="G12" s="10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H12" s="12"/>
     </row>
     <row r="13" spans="2:8" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="4">
@@ -3864,13 +3953,13 @@
         <v>17</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D14" s="4">
         <v>0.3</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F14" s="10"/>
       <c r="G14" s="4"/>
@@ -3881,13 +3970,13 @@
         <v>18</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D15" s="4">
         <v>1.4399999999999999E-5</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="F15" s="10"/>
       <c r="G15" s="10" t="s">
@@ -3900,7 +3989,7 @@
         <v>6</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D16" s="4">
         <v>1.17</v>
@@ -3910,60 +3999,60 @@
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H16" s="12"/>
     </row>
     <row r="17" spans="2:8" ht="67.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="50" t="s">
+      <c r="B17" s="48" t="s">
         <v>13</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D17" s="8">
         <f>(2*D9*Constants!C6)/(Wing!D16*Wing!D12*Wing!D10*Wing!D10)</f>
         <v>0.91637231815803244</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="12"/>
     </row>
     <row r="18" spans="2:8" ht="43.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="50" t="s">
+      <c r="B18" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>31</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>32</v>
       </c>
       <c r="D18" s="9">
         <f>SQRT(D19*D17)</f>
         <v>3.0271642145051074</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="12"/>
     </row>
     <row r="19" spans="2:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="47" t="s">
+      <c r="B19" s="45" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="13" t="s">
         <v>33</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>34</v>
       </c>
       <c r="D19" s="14">
         <v>10</v>
       </c>
       <c r="E19" s="14"/>
       <c r="F19" s="14"/>
-      <c r="G19" s="51" t="s">
-        <v>39</v>
+      <c r="G19" s="49" t="s">
+        <v>37</v>
       </c>
       <c r="H19" s="15"/>
     </row>
@@ -3975,7 +4064,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{189935A4-45F1-46FF-93DA-944832471E2E}">
-  <dimension ref="B1:H20"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
@@ -4009,34 +4098,34 @@
     </row>
     <row r="7" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="43" t="s">
+      <c r="B8" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="44" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="44" t="s">
+      <c r="C8" s="42" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="44" t="s">
+      <c r="E8" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="44" t="s">
+      <c r="F8" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="44" t="s">
+      <c r="G8" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="45" t="s">
+      <c r="H8" s="43" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D9" s="23">
         <v>0.03</v>
@@ -4044,96 +4133,96 @@
       <c r="E9" s="23"/>
       <c r="F9" s="23"/>
       <c r="G9" s="30" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="H9" s="24"/>
     </row>
     <row r="10" spans="2:8" ht="45" x14ac:dyDescent="0.25">
       <c r="B10" s="21" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D10" s="23">
         <v>1</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F10" s="23"/>
       <c r="G10" s="23"/>
       <c r="H10" s="24"/>
     </row>
     <row r="11" spans="2:8" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="46" t="s">
-        <v>45</v>
+      <c r="B11" s="44" t="s">
+        <v>60</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" s="36">
+        <v>43</v>
+      </c>
+      <c r="D11" s="34">
         <f>(D9*D12*D13)/D10</f>
         <v>8.3220284660732544E-2</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="F11" s="23"/>
       <c r="G11" s="23"/>
       <c r="H11" s="24"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="11" t="s">
-        <v>47</v>
+      <c r="B12" s="44" t="s">
+        <v>44</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="D12" s="37">
+        <v>45</v>
+      </c>
+      <c r="D12" s="35">
         <f>Wing!D18</f>
         <v>3.0271642145051074</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F12" s="30"/>
       <c r="G12" s="30"/>
       <c r="H12" s="24"/>
     </row>
-    <row r="13" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="47" t="s">
-        <v>49</v>
+    <row r="13" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="25" t="s">
+        <v>46</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D13" s="32">
         <f>Wing!D17</f>
         <v>0.91637231815803244</v>
       </c>
       <c r="E13" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13" s="48"/>
+        <v>59</v>
+      </c>
+      <c r="F13" s="46"/>
       <c r="G13" s="27"/>
       <c r="H13" s="28"/>
     </row>
     <row r="14" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="38"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="40"/>
-      <c r="G14" s="38"/>
-      <c r="H14" s="38"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="36"/>
     </row>
     <row r="15" spans="2:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="16" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D15" s="19">
         <v>0.5</v>
@@ -4141,91 +4230,98 @@
       <c r="E15" s="18"/>
       <c r="F15" s="18"/>
       <c r="G15" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="H15" s="20"/>
     </row>
     <row r="16" spans="2:8" ht="45" x14ac:dyDescent="0.25">
       <c r="B16" s="21" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D16" s="23">
         <v>1</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F16" s="23"/>
       <c r="G16" s="23"/>
       <c r="H16" s="24"/>
     </row>
-    <row r="17" spans="2:8" ht="48.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="48.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C17" s="31" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D17" s="32">
         <f>(D15*Wing!D14*'V-tail'!D13)/'V-tail'!D16</f>
         <v>0.13745584772370487</v>
       </c>
-      <c r="E17" s="35" t="s">
-        <v>35</v>
+      <c r="E17" s="27" t="s">
+        <v>59</v>
       </c>
       <c r="F17" s="27"/>
       <c r="G17" s="27"/>
       <c r="H17" s="28"/>
     </row>
-    <row r="18" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="38"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="38"/>
-      <c r="H18" s="38"/>
+    <row r="18" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="36"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="36"/>
     </row>
-    <row r="19" spans="2:8" ht="40.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="34" t="s">
-        <v>59</v>
+    <row r="19" spans="1:8" ht="40.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="52" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="50" t="s">
+        <v>56</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D19" s="33">
         <f>DEGREES(ATAN(SQRT(D11/D17)))</f>
         <v>37.886329893038969</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F19" s="18"/>
       <c r="G19" s="18"/>
       <c r="H19" s="20"/>
     </row>
-    <row r="20" spans="2:8" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="25" t="s">
-        <v>60</v>
+    <row r="20" spans="1:8" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="53"/>
+      <c r="B20" s="51" t="s">
+        <v>57</v>
       </c>
       <c r="C20" s="27" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D20" s="32">
         <f>D17+D11</f>
         <v>0.2206761323844374</v>
       </c>
       <c r="E20" s="27" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="F20" s="27"/>
       <c r="G20" s="27"/>
       <c r="H20" s="28"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A19:A20"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Added formulas for Polhamus
</commit_message>
<xml_diff>
--- a/Design_Formulas.xlsx
+++ b/Design_Formulas.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A1097411\Documents\GitHub\ORGOfly-CAD-model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Drones\ORGOfly-CAD-model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47ADB889-0AD4-4C18-8138-B8966D0BDFA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FA68316-25DB-48FA-8138-51A2A436717D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{9597FAC8-E3BA-4239-B29C-D9DA52C8E4BB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{9597FAC8-E3BA-4239-B29C-D9DA52C8E4BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Constants" sheetId="2" r:id="rId1"/>
     <sheet name="Wing" sheetId="1" r:id="rId2"/>
     <sheet name="V-tail" sheetId="3" r:id="rId3"/>
     <sheet name="Fuselage" sheetId="4" r:id="rId4"/>
+    <sheet name="Neutral point" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="117">
   <si>
     <t>kg</t>
   </si>
@@ -640,6 +641,105 @@
   <si>
     <t>Around 25% of the wing chord from the wing tip. Could be calculated at a later stage when the preliminary design is done.</t>
   </si>
+  <si>
+    <t>Fuselage</t>
+  </si>
+  <si>
+    <r>
+      <t>l</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>front</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>l</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>aft</t>
+    </r>
+  </si>
+  <si>
+    <t>Front fuselage</t>
+  </si>
+  <si>
+    <r>
+      <t>l</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>fus</t>
+    </r>
+  </si>
+  <si>
+    <t>Aft fuselage</t>
+  </si>
+  <si>
+    <t>estimated from the right picture (subject  to change)</t>
+  </si>
+  <si>
+    <t>Fuselage lenght</t>
+  </si>
+  <si>
+    <t>From moment lever arm from v-tail</t>
+  </si>
+  <si>
+    <r>
+      <t>d</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>fus</t>
+    </r>
+  </si>
+  <si>
+    <t>Diameter of fuselage</t>
+  </si>
+  <si>
+    <t>from LxWxH (subject to change if too big)</t>
+  </si>
+  <si>
+    <t>Wing contribution</t>
+  </si>
+  <si>
+    <t>Position of Aerodynamic Center</t>
+  </si>
+  <si>
+    <t>Moment Coeff. Of the wing</t>
+  </si>
+  <si>
+    <t>Lift coeff. Depending on the angle of attack</t>
+  </si>
+  <si>
+    <t>polhamus formula</t>
+  </si>
 </sst>
 </file>
 
@@ -649,7 +749,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -702,6 +802,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -735,7 +842,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -995,11 +1102,83 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1149,6 +1328,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -1167,11 +1351,46 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1471,7 +1690,13 @@
                         <a:rPr lang="en-GB" sz="1200" b="0" i="1">
                           <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                         </a:rPr>
-                        <m:t>2∗</m:t>
+                        <m:t>2</m:t>
+                      </m:r>
+                      <m:r>
+                        <a:rPr lang="en-GB" sz="1200" b="0" i="1">
+                          <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        </a:rPr>
+                        <m:t>∗</m:t>
                       </m:r>
                       <m:r>
                         <a:rPr lang="en-GB" sz="1200" b="0" i="1">
@@ -3721,7 +3946,13 @@
                             <a:rPr lang="en-GB" sz="1100" i="1">
                               <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                             </a:rPr>
-                            <m:t>−1</m:t>
+                            <m:t>−</m:t>
+                          </m:r>
+                          <m:r>
+                            <a:rPr lang="en-GB" sz="1100" i="1">
+                              <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            </a:rPr>
+                            <m:t>1</m:t>
                           </m:r>
                         </m:sup>
                       </m:sSup>
@@ -4424,7 +4655,7 @@
     <xdr:to>
       <xdr:col>20</xdr:col>
       <xdr:colOff>503845</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>69138</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -4458,6 +4689,1845 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>320138</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>535727</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1F5FC672-108B-448D-985A-A6D8456530A5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9540338" y="190500"/>
+          <a:ext cx="6921189" cy="4371975"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>120174</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>88455</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="718026" cy="176651"/>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="3" name="TextBox 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0EDCDE1-0BA2-CDE2-4DDB-6AF0AD8E70FD}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="777399" y="2593530"/>
+              <a:ext cx="718026" cy="176651"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1100" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:acc>
+                          <m:accPr>
+                            <m:chr m:val="̅"/>
+                            <m:ctrlPr>
+                              <a:rPr lang="en-US" sz="1100" i="1">
+                                <a:solidFill>
+                                  <a:schemeClr val="tx1"/>
+                                </a:solidFill>
+                                <a:effectLst/>
+                                <a:latin typeface="+mn-lt"/>
+                                <a:ea typeface="+mn-ea"/>
+                                <a:cs typeface="+mn-cs"/>
+                              </a:rPr>
+                            </m:ctrlPr>
+                          </m:accPr>
+                          <m:e>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:solidFill>
+                                  <a:schemeClr val="tx1"/>
+                                </a:solidFill>
+                                <a:effectLst/>
+                                <a:latin typeface="+mn-lt"/>
+                                <a:ea typeface="+mn-ea"/>
+                                <a:cs typeface="+mn-cs"/>
+                              </a:rPr>
+                              <m:t>𝑥</m:t>
+                            </m:r>
+                          </m:e>
+                        </m:acc>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:solidFill>
+                              <a:schemeClr val="tx1"/>
+                            </a:solidFill>
+                            <a:effectLst/>
+                            <a:latin typeface="+mn-lt"/>
+                            <a:ea typeface="+mn-ea"/>
+                            <a:cs typeface="+mn-cs"/>
+                          </a:rPr>
+                          <m:t>𝐴𝐶</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:solidFill>
+                              <a:schemeClr val="tx1"/>
+                            </a:solidFill>
+                            <a:effectLst/>
+                            <a:latin typeface="+mn-lt"/>
+                            <a:ea typeface="+mn-ea"/>
+                            <a:cs typeface="+mn-cs"/>
+                          </a:rPr>
+                          <m:t>,</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:solidFill>
+                              <a:schemeClr val="tx1"/>
+                            </a:solidFill>
+                            <a:effectLst/>
+                            <a:latin typeface="+mn-lt"/>
+                            <a:ea typeface="+mn-ea"/>
+                            <a:cs typeface="+mn-cs"/>
+                          </a:rPr>
+                          <m:t>𝑊</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="3" name="TextBox 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0EDCDE1-0BA2-CDE2-4DDB-6AF0AD8E70FD}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="777399" y="2593530"/>
+              <a:ext cx="718026" cy="176651"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:effectLst/>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:rPr>
+                <a:t>𝑥 ̅</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:effectLst/>
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:rPr>
+                <a:t>_(</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:effectLst/>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:rPr>
+                <a:t>𝐴𝐶,𝑊</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:effectLst/>
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:rPr>
+                <a:t>)</a:t>
+              </a:r>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>333375</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>14287</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1975284" cy="351186"/>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="4" name="TextBox 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00D935CC-4C27-78F0-2278-2BD5BE7C93F3}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="7124700" y="2519362"/>
+              <a:ext cx="1975284" cy="351186"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="bg-BG" sz="1100" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:acc>
+                          <m:accPr>
+                            <m:chr m:val="̅"/>
+                            <m:ctrlPr>
+                              <a:rPr lang="bg-BG" sz="1100" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                            </m:ctrlPr>
+                          </m:accPr>
+                          <m:e>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑥</m:t>
+                            </m:r>
+                          </m:e>
+                        </m:acc>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝐴𝐶</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>,</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑊</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>=</m:t>
+                    </m:r>
+                    <m:f>
+                      <m:fPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:fPr>
+                      <m:num>
+                        <m:sSub>
+                          <m:sSubPr>
+                            <m:ctrlPr>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                            </m:ctrlPr>
+                          </m:sSubPr>
+                          <m:e>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑥</m:t>
+                            </m:r>
+                          </m:e>
+                          <m:sub>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>0</m:t>
+                            </m:r>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>,</m:t>
+                            </m:r>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑊</m:t>
+                            </m:r>
+                          </m:sub>
+                        </m:sSub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>+(</m:t>
+                        </m:r>
+                        <m:sSub>
+                          <m:sSubPr>
+                            <m:ctrlPr>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                            </m:ctrlPr>
+                          </m:sSubPr>
+                          <m:e>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑛</m:t>
+                            </m:r>
+                          </m:e>
+                          <m:sub>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝐴𝐶</m:t>
+                            </m:r>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>,</m:t>
+                            </m:r>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑊</m:t>
+                            </m:r>
+                          </m:sub>
+                        </m:sSub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>∗</m:t>
+                        </m:r>
+                        <m:sSub>
+                          <m:sSubPr>
+                            <m:ctrlPr>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                            </m:ctrlPr>
+                          </m:sSubPr>
+                          <m:e>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑐</m:t>
+                            </m:r>
+                          </m:e>
+                          <m:sub>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑟𝑜𝑜𝑡</m:t>
+                            </m:r>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>,</m:t>
+                            </m:r>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑊</m:t>
+                            </m:r>
+                          </m:sub>
+                        </m:sSub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>)</m:t>
+                        </m:r>
+                      </m:num>
+                      <m:den>
+                        <m:sSub>
+                          <m:sSubPr>
+                            <m:ctrlPr>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                            </m:ctrlPr>
+                          </m:sSubPr>
+                          <m:e>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑐</m:t>
+                            </m:r>
+                          </m:e>
+                          <m:sub>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑀𝐴𝐶</m:t>
+                            </m:r>
+                          </m:sub>
+                        </m:sSub>
+                      </m:den>
+                    </m:f>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="4" name="TextBox 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00D935CC-4C27-78F0-2278-2BD5BE7C93F3}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="7124700" y="2519362"/>
+              <a:ext cx="1975284" cy="351186"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝑥</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="bg-BG" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> ̅_(</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝐴𝐶,𝑊</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="bg-BG" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>)</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>=(𝑥_(0,𝑊)+(𝑛_(𝐴𝐶,𝑊)∗𝑐_(𝑟𝑜𝑜𝑡,𝑊)))/𝑐_𝑀𝐴𝐶 </a:t>
+              </a:r>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>109537</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="830740" cy="176651"/>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="5" name="TextBox 4">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6DE02C36-E9F2-6182-2BB2-7E1C9B780BB0}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4352925" y="2614612"/>
+              <a:ext cx="830740" cy="176651"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="bg-BG" sz="1100" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑛</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝐴𝐶</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>,</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑊</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>=</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>25</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>%</m:t>
+                    </m:r>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="5" name="TextBox 4">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6DE02C36-E9F2-6182-2BB2-7E1C9B780BB0}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4352925" y="2614612"/>
+              <a:ext cx="830740" cy="176651"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝑛</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="bg-BG" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>_(</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝐴𝐶,𝑊</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="bg-BG" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>)</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>=25%</a:t>
+              </a:r>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>90487</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="895350" cy="176651"/>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="6" name="TextBox 5">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBCE2798-42CE-0BC0-6D2A-E1F227C4FC36}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="695325" y="2005012"/>
+              <a:ext cx="895350" cy="176651"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="bg-BG" sz="1100" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝐶</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑀</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝛼</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>,</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑊</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="6" name="TextBox 5">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBCE2798-42CE-0BC0-6D2A-E1F227C4FC36}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="695325" y="2005012"/>
+              <a:ext cx="895350" cy="176651"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝐶</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="bg-BG" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>_(</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝑀</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝛼,𝑊</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="bg-BG" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>)</a:t>
+              </a:r>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>485775</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>109537</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1479892" cy="176651"/>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="7" name="TextBox 6">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9A67F05-2B73-47BD-DCD9-F0453439C37F}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="7277100" y="2024062"/>
+              <a:ext cx="1479892" cy="176651"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="bg-BG" sz="1100" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝐶</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑀</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝛼</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>,</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑊</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>=−</m:t>
+                    </m:r>
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝐶</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝐿</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝛼</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>,</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑊</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>∗</m:t>
+                    </m:r>
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:acc>
+                          <m:accPr>
+                            <m:chr m:val="̅"/>
+                            <m:ctrlPr>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                            </m:ctrlPr>
+                          </m:accPr>
+                          <m:e>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑥</m:t>
+                            </m:r>
+                          </m:e>
+                        </m:acc>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝐴𝐶</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>,</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑊</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="7" name="TextBox 6">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9A67F05-2B73-47BD-DCD9-F0453439C37F}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="7277100" y="2024062"/>
+              <a:ext cx="1479892" cy="176651"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝐶</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="bg-BG" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>_(</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝑀</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝛼,𝑊</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="bg-BG" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>)</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>=−𝐶_(𝐿</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝛼,𝑊)</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>∗𝑥 ̅_(𝐴𝐶,𝑊)</a:t>
+              </a:r>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>185737</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="360099" cy="176651"/>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="8" name="TextBox 7">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69BFB39D-C44A-3CA3-60AB-399BD779004F}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="923925" y="2481262"/>
+              <a:ext cx="360099" cy="176651"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="bg-BG" sz="1100" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝐶</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝐿</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝛼</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>,</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>𝑊</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="8" name="TextBox 7">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69BFB39D-C44A-3CA3-60AB-399BD779004F}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="923925" y="2481262"/>
+              <a:ext cx="360099" cy="176651"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝐶</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="bg-BG" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>_(</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝐿</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>𝛼,𝑊</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="bg-BG" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>)</a:t>
+              </a:r>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>361949</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>184350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>77572</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>19764</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E43F4123-1600-4B68-6085-9DD864FDF715}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9582149" y="4613475"/>
+          <a:ext cx="7030823" cy="3654939"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>598713</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>53563</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>159222</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>183083</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{01C0A1A5-0C11-4AA4-C82C-F3C462A8C6A4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16559892" y="434563"/>
+          <a:ext cx="6296044" cy="3408841"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>179343</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>566188</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="644857" cy="173766"/>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="12" name="TextBox 11">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9ED666B2-4A0F-42F6-FF67-471E7BE3BCBC}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="833669" y="2860471"/>
+              <a:ext cx="644857" cy="173766"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:r>
+                      <m:rPr>
+                        <m:sty m:val="p"/>
+                      </m:rPr>
+                      <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>tan</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>⁡(</m:t>
+                    </m:r>
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:r>
+                          <m:rPr>
+                            <m:sty m:val="p"/>
+                          </m:rPr>
+                          <a:rPr lang="el-GR" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>Λ</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>50</m:t>
+                        </m:r>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>%</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>)</m:t>
+                    </m:r>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="12" name="TextBox 11">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9ED666B2-4A0F-42F6-FF67-471E7BE3BCBC}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="833669" y="2860471"/>
+              <a:ext cx="644857" cy="173766"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>tan⁡(</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="el-GR" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>Λ</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>_(50%))</a:t>
+              </a:r>
+              <a:endParaRPr lang="bg-BG" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -4779,9 +6849,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C4018A4-7FF2-4E68-A485-08C5C78F0065}">
   <dimension ref="B6:D6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>12</v>
       </c>
@@ -4800,19 +6870,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2A91C97-B0A7-4FD8-8682-2CCA08648534}">
   <dimension ref="A1:G24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" customWidth="1"/>
-    <col min="5" max="5" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
-    <col min="7" max="7" width="28.33203125" customWidth="1"/>
-    <col min="9" max="9" width="12.6640625" customWidth="1"/>
+    <col min="7" max="7" width="28.28515625" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="35" t="s">
         <v>53</v>
       </c>
@@ -4820,25 +6890,25 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C7" s="35"/>
     </row>
-    <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="47" t="s">
         <v>9</v>
       </c>
@@ -4858,11 +6928,11 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="65" t="s">
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="68" t="s">
         <v>89</v>
       </c>
-      <c r="B9" s="72" t="s">
+      <c r="B9" s="66" t="s">
         <v>1</v>
       </c>
       <c r="C9" s="40" t="s">
@@ -4877,8 +6947,8 @@
       <c r="F9" s="37"/>
       <c r="G9" s="38"/>
     </row>
-    <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A10" s="66"/>
+    <row r="10" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+      <c r="A10" s="69"/>
       <c r="B10" s="39" t="s">
         <v>52</v>
       </c>
@@ -4892,8 +6962,8 @@
       <c r="F10" s="4"/>
       <c r="G10" s="11"/>
     </row>
-    <row r="11" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A11" s="66"/>
+    <row r="11" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+      <c r="A11" s="69"/>
       <c r="B11" s="39" t="s">
         <v>51</v>
       </c>
@@ -4907,8 +6977,8 @@
       <c r="F11" s="4"/>
       <c r="G11" s="11"/>
     </row>
-    <row r="12" spans="1:7" ht="58.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="66"/>
+    <row r="12" spans="1:7" ht="63" x14ac:dyDescent="0.25">
+      <c r="A12" s="69"/>
       <c r="B12" s="39" t="s">
         <v>20</v>
       </c>
@@ -4924,8 +6994,8 @@
       </c>
       <c r="G12" s="11"/>
     </row>
-    <row r="13" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="66"/>
+    <row r="13" spans="1:7" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="69"/>
       <c r="B13" s="39" t="s">
         <v>19</v>
       </c>
@@ -4942,8 +7012,8 @@
       </c>
       <c r="G13" s="11"/>
     </row>
-    <row r="14" spans="1:7" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="66"/>
+    <row r="14" spans="1:7" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="69"/>
       <c r="B14" s="39" t="s">
         <v>15</v>
       </c>
@@ -4959,8 +7029,8 @@
       <c r="F14" s="4"/>
       <c r="G14" s="11"/>
     </row>
-    <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="66"/>
+    <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="69"/>
       <c r="B15" s="39" t="s">
         <v>16</v>
       </c>
@@ -4978,8 +7048,8 @@
       </c>
       <c r="G15" s="11"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="66"/>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="69"/>
       <c r="B16" s="39" t="s">
         <v>5</v>
       </c>
@@ -4997,9 +7067,9 @@
       </c>
       <c r="G16" s="11"/>
     </row>
-    <row r="17" spans="1:7" ht="67.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="66"/>
-      <c r="B17" s="71" t="s">
+    <row r="17" spans="1:7" ht="67.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="69"/>
+      <c r="B17" s="65" t="s">
         <v>11</v>
       </c>
       <c r="C17" s="7" t="s">
@@ -5015,9 +7085,9 @@
       <c r="F17" s="4"/>
       <c r="G17" s="11"/>
     </row>
-    <row r="18" spans="1:7" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="66"/>
-      <c r="B18" s="71" t="s">
+    <row r="18" spans="1:7" ht="43.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="69"/>
+      <c r="B18" s="65" t="s">
         <v>27</v>
       </c>
       <c r="C18" s="7" t="s">
@@ -5033,8 +7103,8 @@
       <c r="F18" s="4"/>
       <c r="G18" s="11"/>
     </row>
-    <row r="19" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="66"/>
+    <row r="19" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="69"/>
       <c r="B19" s="39" t="s">
         <v>29</v>
       </c>
@@ -5050,8 +7120,8 @@
       </c>
       <c r="G19" s="11"/>
     </row>
-    <row r="20" spans="1:7" ht="44.4" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="67"/>
+    <row r="20" spans="1:7" ht="62.25" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="70"/>
       <c r="B20" s="42" t="s">
         <v>98</v>
       </c>
@@ -5062,19 +7132,19 @@
         <f>0.25*D14</f>
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="E20" s="73" t="s">
+      <c r="E20" s="12" t="s">
         <v>18</v>
       </c>
       <c r="F20" s="34" t="s">
         <v>99</v>
       </c>
-      <c r="G20" s="74" t="s">
+      <c r="G20" s="67" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="65" t="s">
+    <row r="21" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="68" t="s">
         <v>78</v>
       </c>
       <c r="B22" s="45"/>
@@ -5091,8 +7161,8 @@
       <c r="F22" s="37"/>
       <c r="G22" s="38"/>
     </row>
-    <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="66"/>
+    <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="69"/>
       <c r="B23" s="39"/>
       <c r="C23" s="6" t="s">
         <v>80</v>
@@ -5107,8 +7177,8 @@
       <c r="F23" s="4"/>
       <c r="G23" s="11"/>
     </row>
-    <row r="24" spans="1:7" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="67"/>
+    <row r="24" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="70"/>
       <c r="B24" s="42"/>
       <c r="C24" s="43" t="s">
         <v>81</v>
@@ -5138,18 +7208,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{189935A4-45F1-46FF-93DA-944832471E2E}">
   <dimension ref="A1:G29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" style="30" customWidth="1"/>
-    <col min="5" max="5" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" style="30" customWidth="1"/>
+    <col min="5" max="5" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
-    <col min="7" max="7" width="36.44140625" customWidth="1"/>
+    <col min="7" max="7" width="36.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="35" t="s">
         <v>54</v>
       </c>
@@ -5157,23 +7227,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="47" t="s">
         <v>9</v>
       </c>
@@ -5193,8 +7263,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="65" t="s">
+    <row r="9" spans="1:7" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="68" t="s">
         <v>90</v>
       </c>
       <c r="B9" s="58" t="s">
@@ -5212,8 +7282,8 @@
       </c>
       <c r="G9" s="17"/>
     </row>
-    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="66"/>
+    <row r="10" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="69"/>
       <c r="B10" s="50" t="s">
         <v>62</v>
       </c>
@@ -5221,7 +7291,7 @@
         <v>36</v>
       </c>
       <c r="D10" s="19">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E10" s="19" t="s">
         <v>18</v>
@@ -5231,8 +7301,8 @@
       </c>
       <c r="G10" s="20"/>
     </row>
-    <row r="11" spans="1:7" ht="35.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="67"/>
+    <row r="11" spans="1:7" ht="35.450000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="70"/>
       <c r="B11" s="36" t="s">
         <v>63</v>
       </c>
@@ -5241,7 +7311,7 @@
       </c>
       <c r="D11" s="59">
         <f>(D9*D12*D13)/D10</f>
-        <v>8.3220284660732544E-2</v>
+        <v>9.2466982956369487E-2</v>
       </c>
       <c r="E11" s="23" t="s">
         <v>47</v>
@@ -5249,7 +7319,7 @@
       <c r="F11" s="23"/>
       <c r="G11" s="24"/>
     </row>
-    <row r="12" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="18" x14ac:dyDescent="0.25">
       <c r="B12" s="52" t="s">
         <v>64</v>
       </c>
@@ -5266,7 +7336,7 @@
       <c r="F12" s="56"/>
       <c r="G12" s="57"/>
     </row>
-    <row r="13" spans="1:7" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="21" t="s">
         <v>60</v>
       </c>
@@ -5283,15 +7353,15 @@
       <c r="F13" s="23"/>
       <c r="G13" s="24"/>
     </row>
-    <row r="14" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="30"/>
       <c r="C14" s="31"/>
       <c r="E14" s="30"/>
       <c r="F14" s="30"/>
       <c r="G14" s="30"/>
     </row>
-    <row r="15" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="65" t="s">
+    <row r="15" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="68" t="s">
         <v>91</v>
       </c>
       <c r="B15" s="58" t="s">
@@ -5309,8 +7379,8 @@
       </c>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="66"/>
+    <row r="16" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="69"/>
       <c r="B16" s="50" t="s">
         <v>58</v>
       </c>
@@ -5318,7 +7388,7 @@
         <v>40</v>
       </c>
       <c r="D16" s="19">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E16" s="19" t="s">
         <v>18</v>
@@ -5328,8 +7398,8 @@
       </c>
       <c r="G16" s="20"/>
     </row>
-    <row r="17" spans="1:7" ht="48.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="67"/>
+    <row r="17" spans="1:7" ht="48.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="70"/>
       <c r="B17" s="36" t="s">
         <v>59</v>
       </c>
@@ -5338,7 +7408,7 @@
       </c>
       <c r="D17" s="27">
         <f>(D15*Wing!D14*'V-tail'!D13)/'V-tail'!D16</f>
-        <v>0.13745584772370487</v>
+        <v>0.15272871969300542</v>
       </c>
       <c r="E17" s="23" t="s">
         <v>47</v>
@@ -5346,7 +7416,7 @@
       <c r="F17" s="23"/>
       <c r="G17" s="24"/>
     </row>
-    <row r="18" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="30"/>
       <c r="C18" s="32"/>
       <c r="D18" s="33"/>
@@ -5354,8 +7424,8 @@
       <c r="F18" s="30"/>
       <c r="G18" s="30"/>
     </row>
-    <row r="19" spans="1:7" ht="40.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="68" t="s">
+    <row r="19" spans="1:7" ht="40.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="71" t="s">
         <v>92</v>
       </c>
       <c r="B19" s="63" t="s">
@@ -5374,8 +7444,8 @@
       <c r="F19" s="15"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="69"/>
+    <row r="20" spans="1:7" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="72"/>
       <c r="B20" s="60" t="s">
         <v>56</v>
       </c>
@@ -5384,7 +7454,7 @@
       </c>
       <c r="D20" s="61">
         <f>D17+D11</f>
-        <v>0.2206761323844374</v>
+        <v>0.2451957026493749</v>
       </c>
       <c r="E20" s="19" t="s">
         <v>47</v>
@@ -5392,8 +7462,8 @@
       <c r="F20" s="19"/>
       <c r="G20" s="20"/>
     </row>
-    <row r="21" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="69"/>
+    <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="72"/>
       <c r="B21" s="62" t="s">
         <v>29</v>
       </c>
@@ -5409,8 +7479,8 @@
       </c>
       <c r="G21" s="11"/>
     </row>
-    <row r="22" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="69"/>
+    <row r="22" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A22" s="72"/>
       <c r="B22" s="60" t="s">
         <v>66</v>
       </c>
@@ -5419,7 +7489,7 @@
       </c>
       <c r="D22" s="29">
         <f>SQRT(D20*D21)</f>
-        <v>0.93952356518490243</v>
+        <v>0.99034479379532236</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>18</v>
@@ -5427,8 +7497,8 @@
       <c r="F22" s="4"/>
       <c r="G22" s="11"/>
     </row>
-    <row r="23" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="69"/>
+    <row r="23" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A23" s="72"/>
       <c r="B23" s="60" t="s">
         <v>68</v>
       </c>
@@ -5437,7 +7507,7 @@
       </c>
       <c r="D23" s="29">
         <f>D22/D21</f>
-        <v>0.23488089129622561</v>
+        <v>0.24758619844883059</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>18</v>
@@ -5445,8 +7515,8 @@
       <c r="F23" s="4"/>
       <c r="G23" s="11"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="69"/>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="72"/>
       <c r="B24" s="62" t="s">
         <v>70</v>
       </c>
@@ -5462,8 +7532,8 @@
       </c>
       <c r="G24" s="11"/>
     </row>
-    <row r="25" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="70"/>
+    <row r="25" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="73"/>
       <c r="B25" s="64" t="s">
         <v>75</v>
       </c>
@@ -5481,9 +7551,9 @@
       </c>
       <c r="G25" s="13"/>
     </row>
-    <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="27" spans="1:7" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A27" s="68" t="s">
+    <row r="26" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="27" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+      <c r="A27" s="71" t="s">
         <v>83</v>
       </c>
       <c r="B27" s="45" t="s">
@@ -5501,8 +7571,8 @@
       </c>
       <c r="G27" s="38"/>
     </row>
-    <row r="28" spans="1:7" ht="29.4" x14ac:dyDescent="0.35">
-      <c r="A28" s="69"/>
+    <row r="28" spans="1:7" ht="31.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="72"/>
       <c r="B28" s="39" t="s">
         <v>94</v>
       </c>
@@ -5511,7 +7581,7 @@
       </c>
       <c r="D28" s="29">
         <f>0.4*D23</f>
-        <v>9.3952356518490251E-2</v>
+        <v>9.9034479379532248E-2</v>
       </c>
       <c r="E28" s="19" t="s">
         <v>18</v>
@@ -5521,8 +7591,8 @@
       </c>
       <c r="G28" s="11"/>
     </row>
-    <row r="29" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="70"/>
+    <row r="29" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="73"/>
       <c r="B29" s="42"/>
       <c r="C29" s="43" t="s">
         <v>86</v>
@@ -5552,9 +7622,513 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6585412D-E6C6-4698-8307-A04D3DB6C7A6}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38" customWidth="1"/>
+    <col min="7" max="7" width="36.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="35"/>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="30"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="30"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="30"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="30"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D5" s="30"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D6" s="30"/>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="30"/>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="79" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="80" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="81" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="80" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="80" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="82" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="74" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9" s="83" t="s">
+        <v>101</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="D9" s="19">
+        <f>1.5*Wing!D14</f>
+        <v>0.44999999999999996</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="77" t="s">
+        <v>106</v>
+      </c>
+      <c r="G9" s="20"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="75"/>
+      <c r="B10" s="83" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="D10" s="19">
+        <f>3*Wing!D14</f>
+        <v>0.89999999999999991</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="G10" s="20"/>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="76"/>
+      <c r="B11" s="84" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="D11" s="29">
+        <f>D9+D10+Wing!D14</f>
+        <v>1.65</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" s="19"/>
+      <c r="G11" s="20"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="85" t="s">
+        <v>109</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="D12" s="78">
+        <v>0.3</v>
+      </c>
+      <c r="E12" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="77" t="s">
+        <v>111</v>
+      </c>
+      <c r="G12" s="20"/>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="22"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="24"/>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="30"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="68"/>
+      <c r="B15" s="58"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="17"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="69"/>
+      <c r="B16" s="50"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="20"/>
+    </row>
+    <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="70"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="24"/>
+    </row>
+    <row r="18" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="30"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+    </row>
+    <row r="19" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="71"/>
+      <c r="B19" s="63"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="17"/>
+    </row>
+    <row r="20" spans="1:7" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="72"/>
+      <c r="B20" s="60"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="61"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="20"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="72"/>
+      <c r="B21" s="62"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="11"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="72"/>
+      <c r="B22" s="60"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="11"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="72"/>
+      <c r="B23" s="60"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="11"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="72"/>
+      <c r="B24" s="62"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="11"/>
+    </row>
+    <row r="25" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="73"/>
+      <c r="B25" s="64"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="13"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A19:A25"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1379866-2160-4925-834D-A41ED5331C38}">
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38" customWidth="1"/>
+    <col min="7" max="7" width="36.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="35"/>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="30"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="30"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="30"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="30"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D5" s="30"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D6" s="30"/>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="30"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="86" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="88" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="81" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="81" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="81" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="81" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="89" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="90"/>
+      <c r="B9" s="65"/>
+      <c r="C9" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="D9" s="19">
+        <f>(Fuselage!D9+Wing!$D$14*0.25)/Wing!$D$14</f>
+        <v>1.7499999999999998</v>
+      </c>
+      <c r="E9" s="19"/>
+      <c r="F9" s="77"/>
+      <c r="G9" s="19"/>
+    </row>
+    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="90"/>
+      <c r="B10" s="65"/>
+      <c r="C10" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+    </row>
+    <row r="11" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="90"/>
+      <c r="B11" s="60"/>
+      <c r="C11" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="D11" s="29"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="90"/>
+      <c r="B12" s="65"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="78"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="77"/>
+      <c r="G12" s="19"/>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="87"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="61"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="30"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="68"/>
+      <c r="B15" s="58"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="17"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="69"/>
+      <c r="B16" s="50"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="20"/>
+    </row>
+    <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="70"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="24"/>
+    </row>
+    <row r="18" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="30"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="71"/>
+      <c r="B19" s="63"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="17"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="72"/>
+      <c r="B20" s="60"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="61"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="20"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="72"/>
+      <c r="B21" s="62"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="11"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="72"/>
+      <c r="B22" s="60"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="11"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="72"/>
+      <c r="B23" s="60"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="11"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="72"/>
+      <c r="B24" s="62"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="11"/>
+    </row>
+    <row r="25" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="73"/>
+      <c r="B25" s="64"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="13"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A19:A25"/>
+    <mergeCell ref="A8:A12"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated Weight and balance sheet
</commit_message>
<xml_diff>
--- a/Design_Formulas.xlsx
+++ b/Design_Formulas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A1097411\Documents\GitHub\ORGOfly-CAD-model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B9F9BB-205D-438B-809A-CBCDED3938AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08E1E84C-7BDC-4408-9FC3-3CE0D7028582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{9597FAC8-E3BA-4239-B29C-D9DA52C8E4BB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{9597FAC8-E3BA-4239-B29C-D9DA52C8E4BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Constants" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="191">
   <si>
     <t>kg</t>
   </si>
@@ -721,9 +721,6 @@
     </r>
   </si>
   <si>
-    <t>from LxWxH (subject to change if too big)</t>
-  </si>
-  <si>
     <t>Wing contribution</t>
   </si>
   <si>
@@ -1058,10 +1055,96 @@
     <t>CG travel range</t>
   </si>
   <si>
-    <t>Estiamted Weight</t>
-  </si>
-  <si>
-    <t>Outer Dimensions</t>
+    <r>
+      <t>l</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>front</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = 1.5 x wing chord</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>l</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>aft</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = 3 x wing chord</t>
+    </r>
+  </si>
+  <si>
+    <t>from max cargo dimensions
+(subject to change if too big)</t>
+  </si>
+  <si>
+    <t>Height</t>
+  </si>
+  <si>
+    <t>Width</t>
+  </si>
+  <si>
+    <t>Length</t>
+  </si>
+  <si>
+    <t>Estimated Weight (g)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model assumed </t>
+  </si>
+  <si>
+    <t>Turnigy BoltX LiHV 6S 10500mAh 22.8V 80C LiPo Battery Pack w/XT90</t>
+  </si>
+  <si>
+    <t>BrotherHobby Avenger 3120 Motors 500KV FPV Drone Motor</t>
+  </si>
+  <si>
+    <t>Φ37.5</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>22inch</t>
+  </si>
+  <si>
+    <t>FLAME 80A 12S V2.0 Multi-Rotor UAVs ESC</t>
+  </si>
+  <si>
+    <t>Fixed</t>
   </si>
 </sst>
 </file>
@@ -1149,7 +1232,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1186,8 +1269,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="27">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -1559,11 +1654,89 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="131">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1759,9 +1932,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -1795,6 +1965,65 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5047,7 +5276,7 @@
       <xdr:col>14</xdr:col>
       <xdr:colOff>546913</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>121920</xdr:rowOff>
+      <xdr:rowOff>83820</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6634,13 +6863,13 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>179343</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>566188</xdr:rowOff>
+      <xdr:colOff>158176</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>121688</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="644857" cy="173766"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="12" name="TextBox 11">
@@ -6654,7 +6883,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="833669" y="2860471"/>
+              <a:off x="814343" y="3868188"/>
               <a:ext cx="644857" cy="173766"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -6746,7 +6975,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="12" name="TextBox 11">
@@ -6760,7 +6989,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="833669" y="2860471"/>
+              <a:off x="814343" y="3868188"/>
               <a:ext cx="644857" cy="173766"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -6788,6 +7017,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" b="0" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
@@ -11137,6 +11367,55 @@
     </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>159003</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>426819</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>57149</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B7FBB58-2B84-B60A-B919-40159FB0E04A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9324975" y="159003"/>
+          <a:ext cx="5313144" cy="4498721"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -11538,7 +11817,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="90" t="s">
+      <c r="A9" s="89" t="s">
         <v>89</v>
       </c>
       <c r="B9" s="66" t="s">
@@ -11557,7 +11836,7 @@
       <c r="G9" s="38"/>
     </row>
     <row r="10" spans="1:7" ht="18" x14ac:dyDescent="0.35">
-      <c r="A10" s="91"/>
+      <c r="A10" s="90"/>
       <c r="B10" s="39" t="s">
         <v>52</v>
       </c>
@@ -11572,7 +11851,7 @@
       <c r="G10" s="11"/>
     </row>
     <row r="11" spans="1:7" ht="18" x14ac:dyDescent="0.35">
-      <c r="A11" s="91"/>
+      <c r="A11" s="90"/>
       <c r="B11" s="39" t="s">
         <v>51</v>
       </c>
@@ -11587,7 +11866,7 @@
       <c r="G11" s="11"/>
     </row>
     <row r="12" spans="1:7" ht="63" x14ac:dyDescent="0.25">
-      <c r="A12" s="91"/>
+      <c r="A12" s="90"/>
       <c r="B12" s="39" t="s">
         <v>20</v>
       </c>
@@ -11604,7 +11883,7 @@
       <c r="G12" s="11"/>
     </row>
     <row r="13" spans="1:7" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="91"/>
+      <c r="A13" s="90"/>
       <c r="B13" s="65" t="s">
         <v>19</v>
       </c>
@@ -11622,7 +11901,7 @@
       <c r="G13" s="11"/>
     </row>
     <row r="14" spans="1:7" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="91"/>
+      <c r="A14" s="90"/>
       <c r="B14" s="39" t="s">
         <v>15</v>
       </c>
@@ -11639,7 +11918,7 @@
       <c r="G14" s="11"/>
     </row>
     <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="91"/>
+      <c r="A15" s="90"/>
       <c r="B15" s="39" t="s">
         <v>16</v>
       </c>
@@ -11658,7 +11937,7 @@
       <c r="G15" s="11"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="91"/>
+      <c r="A16" s="90"/>
       <c r="B16" s="39" t="s">
         <v>5</v>
       </c>
@@ -11677,7 +11956,7 @@
       <c r="G16" s="11"/>
     </row>
     <row r="17" spans="1:7" ht="67.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="91"/>
+      <c r="A17" s="90"/>
       <c r="B17" s="65" t="s">
         <v>11</v>
       </c>
@@ -11695,7 +11974,7 @@
       <c r="G17" s="11"/>
     </row>
     <row r="18" spans="1:7" ht="43.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="91"/>
+      <c r="A18" s="90"/>
       <c r="B18" s="65" t="s">
         <v>27</v>
       </c>
@@ -11713,7 +11992,7 @@
       <c r="G18" s="11"/>
     </row>
     <row r="19" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A19" s="91"/>
+      <c r="A19" s="90"/>
       <c r="B19" s="39" t="s">
         <v>29</v>
       </c>
@@ -11730,7 +12009,7 @@
       <c r="G19" s="11"/>
     </row>
     <row r="20" spans="1:7" ht="62.25" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="92"/>
+      <c r="A20" s="91"/>
       <c r="B20" s="65" t="s">
         <v>98</v>
       </c>
@@ -11753,7 +12032,7 @@
     </row>
     <row r="21" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="90" t="s">
+      <c r="A22" s="89" t="s">
         <v>78</v>
       </c>
       <c r="B22" s="45"/>
@@ -11771,7 +12050,7 @@
       <c r="G22" s="38"/>
     </row>
     <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="91"/>
+      <c r="A23" s="90"/>
       <c r="B23" s="39"/>
       <c r="C23" s="6" t="s">
         <v>80</v>
@@ -11787,7 +12066,7 @@
       <c r="G23" s="11"/>
     </row>
     <row r="24" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="92"/>
+      <c r="A24" s="91"/>
       <c r="B24" s="42"/>
       <c r="C24" s="43" t="s">
         <v>81</v>
@@ -11873,7 +12152,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="90" t="s">
+      <c r="A9" s="89" t="s">
         <v>90</v>
       </c>
       <c r="B9" s="58" t="s">
@@ -11892,7 +12171,7 @@
       <c r="G9" s="17"/>
     </row>
     <row r="10" spans="1:7" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="91"/>
+      <c r="A10" s="90"/>
       <c r="B10" s="50" t="s">
         <v>62</v>
       </c>
@@ -11911,7 +12190,7 @@
       <c r="G10" s="20"/>
     </row>
     <row r="11" spans="1:7" ht="35.450000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="92"/>
+      <c r="A11" s="91"/>
       <c r="B11" s="36" t="s">
         <v>63</v>
       </c>
@@ -11970,7 +12249,7 @@
       <c r="G14" s="30"/>
     </row>
     <row r="15" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="90" t="s">
+      <c r="A15" s="89" t="s">
         <v>91</v>
       </c>
       <c r="B15" s="58" t="s">
@@ -11989,7 +12268,7 @@
       <c r="G15" s="17"/>
     </row>
     <row r="16" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="91"/>
+      <c r="A16" s="90"/>
       <c r="B16" s="50" t="s">
         <v>58</v>
       </c>
@@ -12008,7 +12287,7 @@
       <c r="G16" s="20"/>
     </row>
     <row r="17" spans="1:7" ht="48.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="92"/>
+      <c r="A17" s="91"/>
       <c r="B17" s="36" t="s">
         <v>59</v>
       </c>
@@ -12034,7 +12313,7 @@
       <c r="G18" s="30"/>
     </row>
     <row r="19" spans="1:7" ht="40.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="93" t="s">
+      <c r="A19" s="92" t="s">
         <v>92</v>
       </c>
       <c r="B19" s="63" t="s">
@@ -12054,7 +12333,7 @@
       <c r="G19" s="17"/>
     </row>
     <row r="20" spans="1:7" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="94"/>
+      <c r="A20" s="93"/>
       <c r="B20" s="60" t="s">
         <v>56</v>
       </c>
@@ -12072,7 +12351,7 @@
       <c r="G20" s="20"/>
     </row>
     <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="94"/>
+      <c r="A21" s="93"/>
       <c r="B21" s="62" t="s">
         <v>29</v>
       </c>
@@ -12089,7 +12368,7 @@
       <c r="G21" s="11"/>
     </row>
     <row r="22" spans="1:7" ht="18" x14ac:dyDescent="0.25">
-      <c r="A22" s="94"/>
+      <c r="A22" s="93"/>
       <c r="B22" s="60" t="s">
         <v>66</v>
       </c>
@@ -12107,7 +12386,7 @@
       <c r="G22" s="11"/>
     </row>
     <row r="23" spans="1:7" ht="18" x14ac:dyDescent="0.25">
-      <c r="A23" s="94"/>
+      <c r="A23" s="93"/>
       <c r="B23" s="60" t="s">
         <v>68</v>
       </c>
@@ -12125,7 +12404,7 @@
       <c r="G23" s="11"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="94"/>
+      <c r="A24" s="93"/>
       <c r="B24" s="62" t="s">
         <v>70</v>
       </c>
@@ -12142,7 +12421,7 @@
       <c r="G24" s="11"/>
     </row>
     <row r="25" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="95"/>
+      <c r="A25" s="94"/>
       <c r="B25" s="64" t="s">
         <v>75</v>
       </c>
@@ -12162,7 +12441,7 @@
     </row>
     <row r="26" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="27" spans="1:7" ht="18" x14ac:dyDescent="0.35">
-      <c r="A27" s="93" t="s">
+      <c r="A27" s="92" t="s">
         <v>83</v>
       </c>
       <c r="B27" s="45" t="s">
@@ -12181,7 +12460,7 @@
       <c r="G27" s="38"/>
     </row>
     <row r="28" spans="1:7" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="94"/>
+      <c r="A28" s="93"/>
       <c r="B28" s="39" t="s">
         <v>94</v>
       </c>
@@ -12201,7 +12480,7 @@
       <c r="G28" s="11"/>
     </row>
     <row r="29" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="95"/>
+      <c r="A29" s="94"/>
       <c r="B29" s="42"/>
       <c r="C29" s="43" t="s">
         <v>86</v>
@@ -12299,7 +12578,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="96" t="s">
+      <c r="A9" s="95" t="s">
         <v>100</v>
       </c>
       <c r="B9" s="86" t="s">
@@ -12318,10 +12597,12 @@
       <c r="F9" s="56" t="s">
         <v>106</v>
       </c>
-      <c r="G9" s="57"/>
+      <c r="G9" s="57" t="s">
+        <v>176</v>
+      </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="97"/>
+    <row r="10" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A10" s="96"/>
       <c r="B10" s="50" t="s">
         <v>102</v>
       </c>
@@ -12338,10 +12619,12 @@
       <c r="F10" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="G10" s="20"/>
+      <c r="G10" s="20" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="97"/>
+      <c r="A11" s="96"/>
       <c r="B11" s="73" t="s">
         <v>104</v>
       </c>
@@ -12359,12 +12642,12 @@
       <c r="G11" s="20"/>
     </row>
     <row r="12" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="98"/>
+      <c r="A12" s="97"/>
       <c r="B12" s="87" t="s">
         <v>109</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D12" s="79">
         <v>0.3</v>
@@ -12373,7 +12656,7 @@
         <v>18</v>
       </c>
       <c r="F12" s="82" t="s">
-        <v>110</v>
+        <v>178</v>
       </c>
       <c r="G12" s="24"/>
     </row>
@@ -12410,7 +12693,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="35" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>3</v>
@@ -12466,131 +12749,131 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="85.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="96" t="s">
-        <v>111</v>
+      <c r="A9" s="95" t="s">
+        <v>110</v>
       </c>
       <c r="B9" s="71"/>
       <c r="C9" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D9" s="15">
         <f>(Fuselage!D9+(Wing!$D$14*0.25))/Wing!$D$14</f>
         <v>1.7499999999999998</v>
       </c>
       <c r="E9" s="61" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F9" s="16"/>
       <c r="G9" s="17"/>
     </row>
     <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="97"/>
+      <c r="A10" s="96"/>
       <c r="B10" s="72"/>
       <c r="C10" s="18" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D10" s="69">
         <f>-D11*D9</f>
         <v>-9.6764591226254897</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F10" s="19"/>
       <c r="G10" s="20"/>
     </row>
     <row r="11" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="A11" s="97"/>
+      <c r="A11" s="96"/>
       <c r="B11" s="73"/>
       <c r="C11" s="18" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D11" s="69">
         <f>(2*(22/7)*Wing!D19)/(2+(SQRT((Wing!D19^2)*('Overall AC'!D13)/'Overall AC'!D14+4)))</f>
         <v>5.529405212928852</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F11" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="G11" s="20" t="s">
         <v>117</v>
-      </c>
-      <c r="G11" s="20" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="97"/>
+      <c r="A12" s="96"/>
       <c r="B12" s="72"/>
       <c r="C12" s="18" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D12" s="69">
         <v>0</v>
       </c>
       <c r="E12" s="19"/>
       <c r="F12" s="18" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G12" s="20"/>
     </row>
     <row r="13" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="97"/>
+      <c r="A13" s="96"/>
       <c r="B13" s="78" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D13" s="61">
         <f>1-(0.07)^2</f>
         <v>0.99509999999999998</v>
       </c>
       <c r="E13" s="61" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G13" s="20"/>
     </row>
     <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="97"/>
+      <c r="A14" s="96"/>
       <c r="B14" s="72" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D14" s="69">
         <f>(1+0.75*D15)^2</f>
         <v>1.1881000000000002</v>
       </c>
       <c r="E14" s="61" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G14" s="20"/>
     </row>
     <row r="15" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="98"/>
+      <c r="A15" s="97"/>
       <c r="B15" s="74" t="s">
+        <v>119</v>
+      </c>
+      <c r="C15" s="22" t="s">
         <v>120</v>
-      </c>
-      <c r="C15" s="22" t="s">
-        <v>121</v>
       </c>
       <c r="D15" s="79">
         <f>(0.12*0.3)/0.3</f>
         <v>0.12</v>
       </c>
       <c r="E15" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="F15" s="26" t="s">
         <v>124</v>
-      </c>
-      <c r="F15" s="26" t="s">
-        <v>125</v>
       </c>
       <c r="G15" s="24"/>
     </row>
@@ -12603,30 +12886,30 @@
       <c r="G16" s="30"/>
     </row>
     <row r="17" spans="1:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="96" t="s">
-        <v>132</v>
+      <c r="A17" s="95" t="s">
+        <v>131</v>
       </c>
       <c r="B17" s="71"/>
       <c r="C17" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D17" s="28">
         <f>(D18+(0.25*'V-tail'!D23))/'V-tail'!D23</f>
         <v>5.9143456312893408</v>
       </c>
       <c r="E17" s="46" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F17" s="16"/>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A18" s="97"/>
+      <c r="A18" s="96"/>
       <c r="B18" s="73" t="s">
+        <v>133</v>
+      </c>
+      <c r="C18" s="18" t="s">
         <v>134</v>
-      </c>
-      <c r="C18" s="18" t="s">
-        <v>135</v>
       </c>
       <c r="D18" s="69">
         <f>Fuselage!D11-'V-tail'!D23</f>
@@ -12636,214 +12919,214 @@
         <v>18</v>
       </c>
       <c r="F18" s="68" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G18" s="20"/>
     </row>
     <row r="19" spans="1:7" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="97"/>
+      <c r="A19" s="96"/>
       <c r="B19" s="72"/>
       <c r="C19" s="18" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D19" s="69">
         <f>-(D20*D21*D22)*D23*D17</f>
         <v>-2.5300219037859915</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F19" s="19"/>
       <c r="G19" s="20"/>
     </row>
     <row r="20" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="97"/>
+      <c r="A20" s="96"/>
       <c r="B20" s="72"/>
       <c r="C20" s="18" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D20" s="69">
         <v>0.9</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F20" s="68" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G20" s="20"/>
     </row>
     <row r="21" spans="1:7" ht="40.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="97"/>
+      <c r="A21" s="96"/>
       <c r="B21" s="72"/>
       <c r="C21" s="18" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D21" s="69">
         <v>0.7</v>
       </c>
       <c r="E21" s="19"/>
       <c r="F21" s="68" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G21" s="20"/>
     </row>
     <row r="22" spans="1:7" ht="47.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="97"/>
+      <c r="A22" s="96"/>
       <c r="B22" s="72"/>
       <c r="C22" s="18" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D22" s="69">
         <f>'V-tail'!D17/Wing!D17</f>
         <v>0.16666666666666669</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F22" s="19"/>
       <c r="G22" s="20"/>
     </row>
     <row r="23" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="A23" s="97"/>
+      <c r="A23" s="96"/>
       <c r="B23" s="73"/>
       <c r="C23" s="18" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D23" s="69">
         <f>(2*(22/7)*'V-tail'!D21)/(2+(SQRT(('V-tail'!D21^2)*('Overall AC'!D25)/'Overall AC'!D26+4)))</f>
         <v>4.0740680719180196</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G23" s="20" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="97"/>
+      <c r="A24" s="96"/>
       <c r="B24" s="72"/>
       <c r="C24" s="18" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D24" s="69">
         <v>0</v>
       </c>
       <c r="E24" s="19"/>
       <c r="F24" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G24" s="20"/>
     </row>
     <row r="25" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="A25" s="97"/>
+      <c r="A25" s="96"/>
       <c r="B25" s="78" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D25" s="61">
         <f>1-(0.07)^2</f>
         <v>0.99509999999999998</v>
       </c>
       <c r="E25" s="61" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G25" s="20"/>
     </row>
     <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="97"/>
+      <c r="A26" s="96"/>
       <c r="B26" s="72" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D26" s="69">
         <f>(1+0.75*D27)^2</f>
         <v>1.1881000000000002</v>
       </c>
       <c r="E26" s="61" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G26" s="20"/>
     </row>
     <row r="27" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="98"/>
+      <c r="A27" s="97"/>
       <c r="B27" s="74" t="s">
+        <v>119</v>
+      </c>
+      <c r="C27" s="22" t="s">
         <v>120</v>
-      </c>
-      <c r="C27" s="22" t="s">
-        <v>121</v>
       </c>
       <c r="D27" s="79">
         <f>(0.12*0.248)/0.248</f>
         <v>0.12</v>
       </c>
       <c r="E27" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="F27" s="26" t="s">
         <v>124</v>
-      </c>
-      <c r="F27" s="26" t="s">
-        <v>125</v>
       </c>
       <c r="G27" s="24"/>
     </row>
     <row r="28" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="29" spans="1:7" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="96" t="s">
-        <v>145</v>
+      <c r="A29" s="95" t="s">
+        <v>144</v>
       </c>
       <c r="B29" s="71"/>
       <c r="C29" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D29" s="80">
         <f>45*((D30*(D31^2)*Fuselage!D11)/Wing!D14*Wing!D17)</f>
         <v>0.20412193386970173</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F29" s="37"/>
       <c r="G29" s="38"/>
     </row>
     <row r="30" spans="1:7" ht="33" x14ac:dyDescent="0.35">
-      <c r="A30" s="97"/>
+      <c r="A30" s="96"/>
       <c r="B30" s="72" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D30" s="4">
         <v>0.01</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G30" s="11"/>
     </row>
     <row r="31" spans="1:7" ht="31.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="97"/>
+      <c r="A31" s="96"/>
       <c r="B31" s="72" t="s">
+        <v>147</v>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>148</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>149</v>
       </c>
       <c r="D31" s="9">
         <f>Fuselage!D12</f>
@@ -12853,14 +13136,14 @@
         <v>18</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G31" s="11"/>
     </row>
     <row r="32" spans="1:7" ht="18" x14ac:dyDescent="0.35">
-      <c r="A32" s="97"/>
+      <c r="A32" s="96"/>
       <c r="B32" s="72" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C32" s="7"/>
       <c r="D32" s="9">
@@ -12868,18 +13151,18 @@
         <v>0.31818181818181812</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="11"/>
     </row>
     <row r="33" spans="1:7" ht="32.25" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="98"/>
+      <c r="A33" s="97"/>
       <c r="B33" s="74" t="s">
+        <v>151</v>
+      </c>
+      <c r="C33" s="43" t="s">
         <v>152</v>
-      </c>
-      <c r="C33" s="43" t="s">
-        <v>153</v>
       </c>
       <c r="D33" s="12">
         <f>Fuselage!D9+Wing!D14*0.25</f>
@@ -12893,30 +13176,30 @@
     </row>
     <row r="34" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="35" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A35" s="99" t="s">
-        <v>156</v>
+      <c r="A35" s="98" t="s">
+        <v>155</v>
       </c>
       <c r="B35" s="71"/>
       <c r="C35" s="14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D35" s="80">
         <f>(D10-D29+D19)/D11+D23</f>
         <v>1.8295946643148437</v>
       </c>
       <c r="E35" s="37" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F35" s="37"/>
       <c r="G35" s="38"/>
     </row>
     <row r="36" spans="1:7" ht="62.25" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="100"/>
+      <c r="A36" s="99"/>
       <c r="B36" s="74" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C36" s="43" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D36" s="81">
         <f>D35*0.3</f>
@@ -12926,7 +13209,7 @@
         <v>18</v>
       </c>
       <c r="F36" s="34" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G36" s="13"/>
     </row>
@@ -12944,146 +13227,301 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F858FC13-65B8-4ADF-8133-431E42F1A0C9}">
-  <dimension ref="B2:D20"/>
+  <dimension ref="B1:H22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8" style="113" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="64" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B2" s="4"/>
-      <c r="C2" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>178</v>
+    <row r="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B1" s="129" t="s">
+        <v>190</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="89" t="s">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="130" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="103"/>
+      <c r="C4" s="108" t="s">
+        <v>182</v>
+      </c>
+      <c r="D4" s="117" t="s">
+        <v>179</v>
+      </c>
+      <c r="E4" s="102" t="s">
+        <v>180</v>
+      </c>
+      <c r="F4" s="118" t="s">
+        <v>181</v>
+      </c>
+      <c r="G4" s="108" t="s">
+        <v>187</v>
+      </c>
+      <c r="H4" s="123" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="104" t="s">
+        <v>160</v>
+      </c>
+      <c r="C5" s="109">
+        <v>1150</v>
+      </c>
+      <c r="D5" s="119">
+        <v>66</v>
+      </c>
+      <c r="E5" s="101">
+        <v>48</v>
+      </c>
+      <c r="F5" s="120">
+        <v>175</v>
+      </c>
+      <c r="G5" s="114">
+        <v>2</v>
+      </c>
+      <c r="H5" s="124" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="105" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
+      <c r="C6" s="111">
+        <v>142.69999999999999</v>
+      </c>
+      <c r="D6" s="121">
+        <v>53.2</v>
+      </c>
+      <c r="E6" s="100" t="s">
+        <v>186</v>
+      </c>
+      <c r="F6" s="116"/>
+      <c r="G6" s="110">
+        <v>4</v>
+      </c>
+      <c r="H6" s="125" t="s">
+        <v>185</v>
+      </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B4" s="89" t="s">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="105" t="s">
         <v>162</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="C7" s="111">
+        <v>180</v>
+      </c>
+      <c r="D7" s="127" t="s">
+        <v>188</v>
+      </c>
+      <c r="E7" s="107"/>
+      <c r="F7" s="128"/>
+      <c r="G7" s="110">
+        <v>4</v>
+      </c>
+      <c r="H7" s="125"/>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B5" s="89" t="s">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="105" t="s">
         <v>163</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="C8" s="111">
+        <v>110</v>
+      </c>
+      <c r="D8" s="121">
+        <v>19.5</v>
+      </c>
+      <c r="E8" s="4">
+        <v>35.5</v>
+      </c>
+      <c r="F8" s="11">
+        <v>84</v>
+      </c>
+      <c r="G8" s="110">
+        <v>4</v>
+      </c>
+      <c r="H8" s="125" t="s">
+        <v>189</v>
+      </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="89" t="s">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="105" t="s">
         <v>164</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
+      <c r="C9" s="111"/>
+      <c r="D9" s="121"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="110"/>
+      <c r="H9" s="125"/>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="89" t="s">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="105" t="s">
         <v>165</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="C10" s="111"/>
+      <c r="D10" s="121"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="110">
+        <v>1</v>
+      </c>
+      <c r="H10" s="125"/>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B8" s="89" t="s">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="105" t="s">
         <v>166</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="C11" s="111">
+        <v>3000</v>
+      </c>
+      <c r="D11" s="121"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="110">
+        <v>1</v>
+      </c>
+      <c r="H11" s="125"/>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B9" s="89" t="s">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B12" s="105" t="s">
         <v>167</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="C12" s="111"/>
+      <c r="D12" s="121"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="110"/>
+      <c r="H12" s="125"/>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B10" s="89" t="s">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="105" t="s">
         <v>168</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
+      <c r="C13" s="111"/>
+      <c r="D13" s="121"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="110">
+        <v>1</v>
+      </c>
+      <c r="H13" s="125"/>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B11" s="89" t="s">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="105" t="s">
         <v>169</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="C14" s="111"/>
+      <c r="D14" s="121"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="110">
+        <v>1</v>
+      </c>
+      <c r="H14" s="125"/>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B12" s="89" t="s">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="105" t="s">
         <v>170</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
+      <c r="C15" s="111"/>
+      <c r="D15" s="121"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="110">
+        <v>1</v>
+      </c>
+      <c r="H15" s="125"/>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B13" s="89" t="s">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="105" t="s">
         <v>171</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
+      <c r="C16" s="111"/>
+      <c r="D16" s="121"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="110"/>
+      <c r="H16" s="125"/>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B14" s="89" t="s">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="105"/>
+      <c r="C17" s="111"/>
+      <c r="D17" s="121"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="110"/>
+      <c r="H17" s="125"/>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="105" t="s">
         <v>172</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
+      <c r="C18" s="111"/>
+      <c r="D18" s="121"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="110"/>
+      <c r="H18" s="125"/>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="105"/>
+      <c r="C19" s="111"/>
+      <c r="D19" s="121"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="110"/>
+      <c r="H19" s="125"/>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="4" t="s">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="105" t="s">
         <v>173</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
+      <c r="C20" s="111"/>
+      <c r="D20" s="121"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="110"/>
+      <c r="H20" s="125"/>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="89"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="105" t="s">
+        <v>174</v>
+      </c>
+      <c r="C21" s="111"/>
+      <c r="D21" s="121"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="110"/>
+      <c r="H21" s="125"/>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="89" t="s">
-        <v>174</v>
-      </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B19" s="89" t="s">
+    <row r="22" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="106" t="s">
         <v>175</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B20" s="89" t="s">
-        <v>176</v>
-      </c>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
+      <c r="C22" s="112"/>
+      <c r="D22" s="122"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="115"/>
+      <c r="H22" s="126"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E6:F6"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Created a body shell with holes for wing and vtail
</commit_message>
<xml_diff>
--- a/Design_Formulas.xlsx
+++ b/Design_Formulas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A1097411\Documents\GitHub\ORGOfly-CAD-model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Drones\ORGOfly-CAD-model\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02002259-6CDD-402B-985A-F138DDD3CF16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{9597FAC8-E3BA-4239-B29C-D9DA52C8E4BB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{9597FAC8-E3BA-4239-B29C-D9DA52C8E4BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Constants" sheetId="2" r:id="rId1"/>
@@ -2177,6 +2177,42 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -2221,42 +2257,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -11936,9 +11936,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C4018A4-7FF2-4E68-A485-08C5C78F0065}">
   <dimension ref="B6:D6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>12</v>
       </c>
@@ -11957,19 +11957,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2A91C97-B0A7-4FD8-8682-2CCA08648534}">
   <dimension ref="A1:G24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" customWidth="1"/>
-    <col min="5" max="5" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
-    <col min="7" max="7" width="28.33203125" customWidth="1"/>
-    <col min="9" max="9" width="12.6640625" customWidth="1"/>
+    <col min="7" max="7" width="28.28515625" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>53</v>
       </c>
@@ -11977,25 +11977,25 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C7" s="12"/>
     </row>
-    <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="17" t="s">
         <v>9</v>
       </c>
@@ -12015,8 +12015,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="127" t="s">
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="139" t="s">
         <v>89</v>
       </c>
       <c r="B9" s="55" t="s">
@@ -12034,8 +12034,8 @@
       <c r="F9" s="91"/>
       <c r="G9" s="13"/>
     </row>
-    <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="128"/>
+    <row r="10" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A10" s="140"/>
       <c r="B10" s="52" t="s">
         <v>52</v>
       </c>
@@ -12049,8 +12049,8 @@
       <c r="F10" s="92"/>
       <c r="G10" s="6"/>
     </row>
-    <row r="11" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="128"/>
+    <row r="11" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A11" s="140"/>
       <c r="B11" s="52" t="s">
         <v>51</v>
       </c>
@@ -12064,8 +12064,8 @@
       <c r="F11" s="92"/>
       <c r="G11" s="6"/>
     </row>
-    <row r="12" spans="1:7" ht="58.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="128"/>
+    <row r="12" spans="1:7" ht="63" x14ac:dyDescent="0.25">
+      <c r="A12" s="140"/>
       <c r="B12" s="52" t="s">
         <v>20</v>
       </c>
@@ -12081,8 +12081,8 @@
       </c>
       <c r="G12" s="6"/>
     </row>
-    <row r="13" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="128"/>
+    <row r="13" spans="1:7" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="140"/>
       <c r="B13" s="53" t="s">
         <v>19</v>
       </c>
@@ -12099,8 +12099,8 @@
       </c>
       <c r="G13" s="6"/>
     </row>
-    <row r="14" spans="1:7" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="128"/>
+    <row r="14" spans="1:7" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="140"/>
       <c r="B14" s="52" t="s">
         <v>15</v>
       </c>
@@ -12116,8 +12116,8 @@
       <c r="F14" s="92"/>
       <c r="G14" s="6"/>
     </row>
-    <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="128"/>
+    <row r="15" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="140"/>
       <c r="B15" s="52" t="s">
         <v>16</v>
       </c>
@@ -12135,8 +12135,8 @@
       </c>
       <c r="G15" s="6"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="128"/>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="140"/>
       <c r="B16" s="52" t="s">
         <v>5</v>
       </c>
@@ -12154,8 +12154,8 @@
       </c>
       <c r="G16" s="6"/>
     </row>
-    <row r="17" spans="1:7" ht="67.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="128"/>
+    <row r="17" spans="1:7" ht="67.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="140"/>
       <c r="B17" s="53" t="s">
         <v>11</v>
       </c>
@@ -12172,8 +12172,8 @@
       <c r="F17" s="92"/>
       <c r="G17" s="6"/>
     </row>
-    <row r="18" spans="1:7" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="128"/>
+    <row r="18" spans="1:7" ht="43.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="140"/>
       <c r="B18" s="53" t="s">
         <v>27</v>
       </c>
@@ -12190,8 +12190,8 @@
       <c r="F18" s="92"/>
       <c r="G18" s="6"/>
     </row>
-    <row r="19" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="128"/>
+    <row r="19" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="140"/>
       <c r="B19" s="52" t="s">
         <v>29</v>
       </c>
@@ -12207,8 +12207,8 @@
       </c>
       <c r="G19" s="6"/>
     </row>
-    <row r="20" spans="1:7" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="129"/>
+    <row r="20" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="141"/>
       <c r="B20" s="53" t="s">
         <v>98</v>
       </c>
@@ -12229,14 +12229,14 @@
         <v>96</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C21" s="61"/>
       <c r="D21" s="61"/>
       <c r="E21" s="61"/>
       <c r="F21" s="95"/>
     </row>
-    <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="127" t="s">
+    <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="139" t="s">
         <v>78</v>
       </c>
       <c r="B22" s="16"/>
@@ -12253,8 +12253,8 @@
       <c r="F22" s="91"/>
       <c r="G22" s="13"/>
     </row>
-    <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="128"/>
+    <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="140"/>
       <c r="B23" s="14"/>
       <c r="C23" s="66" t="s">
         <v>80</v>
@@ -12269,8 +12269,8 @@
       <c r="F23" s="92"/>
       <c r="G23" s="6"/>
     </row>
-    <row r="24" spans="1:7" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="129"/>
+    <row r="24" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="141"/>
       <c r="B24" s="15"/>
       <c r="C24" s="67" t="s">
         <v>81</v>
@@ -12300,18 +12300,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{189935A4-45F1-46FF-93DA-944832471E2E}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" style="11" customWidth="1"/>
-    <col min="5" max="5" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" style="11" customWidth="1"/>
+    <col min="5" max="5" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
-    <col min="7" max="7" width="36.44140625" customWidth="1"/>
+    <col min="7" max="7" width="36.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>54</v>
       </c>
@@ -12319,23 +12319,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="17" t="s">
         <v>9</v>
       </c>
@@ -12355,8 +12355,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="127" t="s">
+    <row r="9" spans="1:7" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="139" t="s">
         <v>90</v>
       </c>
       <c r="B9" s="68" t="s">
@@ -12369,13 +12369,13 @@
         <v>0.03</v>
       </c>
       <c r="E9" s="56"/>
-      <c r="F9" s="149" t="s">
+      <c r="F9" s="129" t="s">
         <v>42</v>
       </c>
       <c r="G9" s="8"/>
     </row>
-    <row r="10" spans="1:7" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="128"/>
+    <row r="10" spans="1:7" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="140"/>
       <c r="B10" s="69" t="s">
         <v>62</v>
       </c>
@@ -12388,13 +12388,13 @@
       <c r="E10" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="150" t="s">
+      <c r="F10" s="130" t="s">
         <v>77</v>
       </c>
       <c r="G10" s="9"/>
     </row>
-    <row r="11" spans="1:7" ht="35.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="129"/>
+    <row r="11" spans="1:7" ht="35.450000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="141"/>
       <c r="B11" s="70" t="s">
         <v>63</v>
       </c>
@@ -12408,10 +12408,10 @@
       <c r="E11" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="151"/>
+      <c r="F11" s="131"/>
       <c r="G11" s="10"/>
     </row>
-    <row r="12" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="18" x14ac:dyDescent="0.25">
       <c r="B12" s="73" t="s">
         <v>64</v>
       </c>
@@ -12425,10 +12425,10 @@
       <c r="E12" s="76" t="s">
         <v>18</v>
       </c>
-      <c r="F12" s="152"/>
+      <c r="F12" s="132"/>
       <c r="G12" s="21"/>
     </row>
-    <row r="13" spans="1:7" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="77" t="s">
         <v>60</v>
       </c>
@@ -12442,19 +12442,19 @@
       <c r="E13" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="F13" s="151"/>
+      <c r="F13" s="131"/>
       <c r="G13" s="10"/>
     </row>
-    <row r="14" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="61"/>
       <c r="C14" s="46"/>
       <c r="D14" s="61"/>
       <c r="E14" s="61"/>
-      <c r="F14" s="153"/>
+      <c r="F14" s="133"/>
       <c r="G14" s="11"/>
     </row>
-    <row r="15" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="133" t="s">
+    <row r="15" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="145" t="s">
         <v>91</v>
       </c>
       <c r="B15" s="85" t="s">
@@ -12467,13 +12467,13 @@
         <v>0.5</v>
       </c>
       <c r="E15" s="56"/>
-      <c r="F15" s="149" t="s">
+      <c r="F15" s="129" t="s">
         <v>42</v>
       </c>
       <c r="G15" s="8"/>
     </row>
-    <row r="16" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="134"/>
+    <row r="16" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="146"/>
       <c r="B16" s="52" t="s">
         <v>58</v>
       </c>
@@ -12486,13 +12486,13 @@
       <c r="E16" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="150" t="s">
+      <c r="F16" s="130" t="s">
         <v>77</v>
       </c>
       <c r="G16" s="9"/>
     </row>
-    <row r="17" spans="1:7" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="134"/>
+    <row r="17" spans="1:7" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="146"/>
       <c r="B17" s="53" t="s">
         <v>59</v>
       </c>
@@ -12506,11 +12506,11 @@
       <c r="E17" s="57" t="s">
         <v>47</v>
       </c>
-      <c r="F17" s="150"/>
+      <c r="F17" s="130"/>
       <c r="G17" s="9"/>
     </row>
-    <row r="18" spans="1:7" ht="48.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="135"/>
+    <row r="18" spans="1:7" ht="48.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="147"/>
       <c r="B18" s="101" t="s">
         <v>195</v>
       </c>
@@ -12523,19 +12523,19 @@
       <c r="E18" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="151"/>
+      <c r="F18" s="131"/>
       <c r="G18" s="10"/>
     </row>
-    <row r="19" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="61"/>
       <c r="C19" s="47"/>
       <c r="D19" s="80"/>
       <c r="E19" s="61"/>
-      <c r="F19" s="153"/>
+      <c r="F19" s="133"/>
       <c r="G19" s="11"/>
     </row>
-    <row r="20" spans="1:7" ht="40.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="130" t="s">
+    <row r="20" spans="1:7" ht="40.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="142" t="s">
         <v>92</v>
       </c>
       <c r="B20" s="81" t="s">
@@ -12544,20 +12544,20 @@
       <c r="C20" s="64" t="s">
         <v>43</v>
       </c>
-      <c r="D20" s="147">
+      <c r="D20" s="127">
         <f>DEGREES(ATAN(SQRT(D11/D17)))</f>
         <v>37.886329893038969</v>
       </c>
       <c r="E20" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="F20" s="148" t="s">
+      <c r="F20" s="128" t="s">
         <v>199</v>
       </c>
       <c r="G20" s="8"/>
     </row>
-    <row r="21" spans="1:7" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="131"/>
+    <row r="21" spans="1:7" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="143"/>
       <c r="B21" s="53" t="s">
         <v>56</v>
       </c>
@@ -12571,11 +12571,11 @@
       <c r="E21" s="57" t="s">
         <v>47</v>
       </c>
-      <c r="F21" s="150"/>
+      <c r="F21" s="130"/>
       <c r="G21" s="9"/>
     </row>
-    <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="131"/>
+    <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="143"/>
       <c r="B22" s="52" t="s">
         <v>29</v>
       </c>
@@ -12591,8 +12591,8 @@
       </c>
       <c r="G22" s="6"/>
     </row>
-    <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="131"/>
+    <row r="23" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="143"/>
       <c r="B23" s="53" t="s">
         <v>66</v>
       </c>
@@ -12611,8 +12611,8 @@
       </c>
       <c r="G23" s="6"/>
     </row>
-    <row r="24" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="131"/>
+    <row r="24" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A24" s="143"/>
       <c r="B24" s="53" t="s">
         <v>68</v>
       </c>
@@ -12626,11 +12626,11 @@
       <c r="E24" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="F24" s="150"/>
+      <c r="F24" s="130"/>
       <c r="G24" s="6"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="131"/>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="143"/>
       <c r="B25" s="52" t="s">
         <v>70</v>
       </c>
@@ -12641,13 +12641,13 @@
         <v>0</v>
       </c>
       <c r="E25" s="57"/>
-      <c r="F25" s="150" t="s">
+      <c r="F25" s="130" t="s">
         <v>71</v>
       </c>
       <c r="G25" s="6"/>
     </row>
-    <row r="26" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="132"/>
+    <row r="26" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="144"/>
       <c r="B26" s="84" t="s">
         <v>75</v>
       </c>
@@ -12665,15 +12665,15 @@
       </c>
       <c r="G26" s="7"/>
     </row>
-    <row r="27" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
       <c r="D27" s="61"/>
       <c r="E27" s="61"/>
-      <c r="F27" s="153"/>
+      <c r="F27" s="133"/>
     </row>
-    <row r="28" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="130" t="s">
+    <row r="28" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A28" s="142" t="s">
         <v>83</v>
       </c>
       <c r="B28" s="85" t="s">
@@ -12686,13 +12686,13 @@
       <c r="E28" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="F28" s="148" t="s">
+      <c r="F28" s="128" t="s">
         <v>88</v>
       </c>
       <c r="G28" s="13"/>
     </row>
-    <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A29" s="131"/>
+    <row r="29" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="143"/>
       <c r="B29" s="52" t="s">
         <v>94</v>
       </c>
@@ -12711,8 +12711,8 @@
       </c>
       <c r="G29" s="6"/>
     </row>
-    <row r="30" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="132"/>
+    <row r="30" spans="1:7" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="144"/>
       <c r="B30" s="84"/>
       <c r="C30" s="67" t="s">
         <v>86</v>
@@ -12743,52 +12743,52 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6585412D-E6C6-4698-8307-A04D3DB6C7A6}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" customWidth="1"/>
-    <col min="5" max="5" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
-    <col min="7" max="7" width="36.44140625" customWidth="1"/>
+    <col min="7" max="7" width="36.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12"/>
       <c r="B1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="11"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D2" s="11"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="11"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="11"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D5" s="11"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D6" s="11"/>
     </row>
-    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D7" s="11"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="48"/>
       <c r="B8" s="49" t="s">
         <v>9</v>
@@ -12809,8 +12809,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="136" t="s">
+    <row r="9" spans="1:7" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="148" t="s">
         <v>100</v>
       </c>
       <c r="B9" s="52" t="s">
@@ -12833,8 +12833,8 @@
         <v>169</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="134"/>
+    <row r="10" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A10" s="146"/>
       <c r="B10" s="52" t="s">
         <v>102</v>
       </c>
@@ -12855,8 +12855,8 @@
         <v>170</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="134"/>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="146"/>
       <c r="B11" s="53" t="s">
         <v>104</v>
       </c>
@@ -12873,8 +12873,8 @@
       <c r="F11" s="92"/>
       <c r="G11" s="9"/>
     </row>
-    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="134"/>
+    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="146"/>
       <c r="B12" s="52" t="s">
         <v>108</v>
       </c>
@@ -12892,8 +12892,8 @@
       </c>
       <c r="G12" s="9"/>
     </row>
-    <row r="13" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="135"/>
+    <row r="13" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="147"/>
       <c r="B13" s="54" t="s">
         <v>192</v>
       </c>
@@ -12923,18 +12923,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1379866-2160-4925-834D-A41ED5331C38}">
   <dimension ref="A1:G36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" customWidth="1"/>
-    <col min="5" max="5" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
-    <col min="7" max="7" width="41.5546875" customWidth="1"/>
+    <col min="7" max="7" width="41.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>111</v>
       </c>
@@ -12943,34 +12943,34 @@
       </c>
       <c r="D1" s="11"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D2" s="11"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="11"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="11"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D5" s="11"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D6" s="11"/>
     </row>
-    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D7" s="11"/>
     </row>
-    <row r="8" spans="1:7" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="22"/>
       <c r="B8" s="23" t="s">
         <v>9</v>
@@ -12991,8 +12991,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="137" t="s">
+    <row r="9" spans="1:7" ht="85.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="149" t="s">
         <v>109</v>
       </c>
       <c r="B9" s="86"/>
@@ -13009,8 +13009,8 @@
       <c r="F9" s="96"/>
       <c r="G9" s="8"/>
     </row>
-    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="138"/>
+    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="150"/>
       <c r="B10" s="87"/>
       <c r="C10" s="66" t="s">
         <v>113</v>
@@ -13025,8 +13025,8 @@
       <c r="F10" s="92"/>
       <c r="G10" s="9"/>
     </row>
-    <row r="11" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="138"/>
+    <row r="11" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="150"/>
       <c r="B11" s="87"/>
       <c r="C11" s="66" t="s">
         <v>117</v>
@@ -13045,8 +13045,8 @@
         <v>116</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="138"/>
+    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="150"/>
       <c r="B12" s="87"/>
       <c r="C12" s="66" t="s">
         <v>110</v>
@@ -13060,8 +13060,8 @@
       </c>
       <c r="G12" s="9"/>
     </row>
-    <row r="13" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="138"/>
+    <row r="13" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="150"/>
       <c r="B13" s="88" t="s">
         <v>125</v>
       </c>
@@ -13080,8 +13080,8 @@
       </c>
       <c r="G13" s="9"/>
     </row>
-    <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="138"/>
+    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="150"/>
       <c r="B14" s="87" t="s">
         <v>124</v>
       </c>
@@ -13100,8 +13100,8 @@
       </c>
       <c r="G14" s="9"/>
     </row>
-    <row r="15" spans="1:7" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="139"/>
+    <row r="15" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="151"/>
       <c r="B15" s="70" t="s">
         <v>118</v>
       </c>
@@ -13120,7 +13120,7 @@
       </c>
       <c r="G15" s="10"/>
     </row>
-    <row r="16" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="61"/>
       <c r="C16" s="46"/>
       <c r="D16" s="61"/>
@@ -13128,8 +13128,8 @@
       <c r="F16" s="95"/>
       <c r="G16" s="11"/>
     </row>
-    <row r="17" spans="1:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="137" t="s">
+    <row r="17" spans="1:7" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="149" t="s">
         <v>130</v>
       </c>
       <c r="B17" s="86"/>
@@ -13146,8 +13146,8 @@
       <c r="F17" s="96"/>
       <c r="G17" s="8"/>
     </row>
-    <row r="18" spans="1:7" ht="72" x14ac:dyDescent="0.3">
-      <c r="A18" s="138"/>
+    <row r="18" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A18" s="150"/>
       <c r="B18" s="87" t="s">
         <v>132</v>
       </c>
@@ -13166,8 +13166,8 @@
       </c>
       <c r="G18" s="9"/>
     </row>
-    <row r="19" spans="1:7" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="138"/>
+    <row r="19" spans="1:7" ht="55.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="150"/>
       <c r="B19" s="87"/>
       <c r="C19" s="66" t="s">
         <v>135</v>
@@ -13182,8 +13182,8 @@
       <c r="F19" s="92"/>
       <c r="G19" s="9"/>
     </row>
-    <row r="20" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="138"/>
+    <row r="20" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="150"/>
       <c r="B20" s="87"/>
       <c r="C20" s="66" t="s">
         <v>139</v>
@@ -13199,8 +13199,8 @@
       </c>
       <c r="G20" s="9"/>
     </row>
-    <row r="21" spans="1:7" ht="40.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="138"/>
+    <row r="21" spans="1:7" ht="40.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="150"/>
       <c r="B21" s="87"/>
       <c r="C21" s="66" t="s">
         <v>140</v>
@@ -13214,8 +13214,8 @@
       </c>
       <c r="G21" s="9"/>
     </row>
-    <row r="22" spans="1:7" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="138"/>
+    <row r="22" spans="1:7" ht="47.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="150"/>
       <c r="B22" s="87"/>
       <c r="C22" s="66" t="s">
         <v>141</v>
@@ -13230,8 +13230,8 @@
       <c r="F22" s="92"/>
       <c r="G22" s="9"/>
     </row>
-    <row r="23" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="138"/>
+    <row r="23" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23" s="150"/>
       <c r="B23" s="87"/>
       <c r="C23" s="66" t="s">
         <v>136</v>
@@ -13250,8 +13250,8 @@
         <v>116</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A24" s="138"/>
+    <row r="24" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="150"/>
       <c r="B24" s="87"/>
       <c r="C24" s="66" t="s">
         <v>110</v>
@@ -13265,8 +13265,8 @@
       </c>
       <c r="G24" s="9"/>
     </row>
-    <row r="25" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="138"/>
+    <row r="25" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A25" s="150"/>
       <c r="B25" s="88" t="s">
         <v>125</v>
       </c>
@@ -13285,8 +13285,8 @@
       </c>
       <c r="G25" s="9"/>
     </row>
-    <row r="26" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="138"/>
+    <row r="26" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="150"/>
       <c r="B26" s="87" t="s">
         <v>124</v>
       </c>
@@ -13305,8 +13305,8 @@
       </c>
       <c r="G26" s="9"/>
     </row>
-    <row r="27" spans="1:7" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="139"/>
+    <row r="27" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="151"/>
       <c r="B27" s="70" t="s">
         <v>118</v>
       </c>
@@ -13325,15 +13325,15 @@
       </c>
       <c r="G27" s="10"/>
     </row>
-    <row r="28" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="61"/>
       <c r="C28" s="61"/>
       <c r="D28" s="61"/>
       <c r="E28" s="61"/>
       <c r="F28" s="95"/>
     </row>
-    <row r="29" spans="1:7" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="137" t="s">
+    <row r="29" spans="1:7" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="149" t="s">
         <v>143</v>
       </c>
       <c r="B29" s="86"/>
@@ -13350,8 +13350,8 @@
       <c r="F29" s="91"/>
       <c r="G29" s="13"/>
     </row>
-    <row r="30" spans="1:7" ht="30" x14ac:dyDescent="0.3">
-      <c r="A30" s="138"/>
+    <row r="30" spans="1:7" ht="33" x14ac:dyDescent="0.25">
+      <c r="A30" s="150"/>
       <c r="B30" s="87" t="s">
         <v>145</v>
       </c>
@@ -13369,8 +13369,8 @@
       </c>
       <c r="G30" s="6"/>
     </row>
-    <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A31" s="138"/>
+    <row r="31" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="150"/>
       <c r="B31" s="87" t="s">
         <v>146</v>
       </c>
@@ -13389,8 +13389,8 @@
       </c>
       <c r="G31" s="6"/>
     </row>
-    <row r="32" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="138"/>
+    <row r="32" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A32" s="150"/>
       <c r="B32" s="87" t="s">
         <v>149</v>
       </c>
@@ -13405,8 +13405,8 @@
       <c r="F32" s="92"/>
       <c r="G32" s="6"/>
     </row>
-    <row r="33" spans="1:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="139"/>
+    <row r="33" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="151"/>
       <c r="B33" s="70" t="s">
         <v>150</v>
       </c>
@@ -13423,15 +13423,15 @@
       <c r="F33" s="97"/>
       <c r="G33" s="7"/>
     </row>
-    <row r="34" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="61"/>
       <c r="C34" s="61"/>
       <c r="D34" s="61"/>
       <c r="E34" s="61"/>
       <c r="F34" s="95"/>
     </row>
-    <row r="35" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="140" t="s">
+    <row r="35" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A35" s="152" t="s">
         <v>154</v>
       </c>
       <c r="B35" s="86"/>
@@ -13448,8 +13448,8 @@
       <c r="F35" s="91"/>
       <c r="G35" s="13"/>
     </row>
-    <row r="36" spans="1:7" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="141"/>
+    <row r="36" spans="1:7" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="153"/>
       <c r="B36" s="70" t="s">
         <v>155</v>
       </c>
@@ -13483,26 +13483,26 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F858FC13-65B8-4ADF-8133-431E42F1A0C9}">
   <dimension ref="B1:J22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" customWidth="1"/>
-    <col min="5" max="5" width="6.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" customWidth="1"/>
+    <col min="5" max="5" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8" style="34" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="64" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B1" s="42"/>
     </row>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B2" s="43"/>
     </row>
-    <row r="3" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="27"/>
       <c r="C4" s="30" t="s">
         <v>175</v>
@@ -13529,7 +13529,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" s="28" t="s">
         <v>159</v>
       </c>
@@ -13552,7 +13552,7 @@
       <c r="I5" s="123"/>
       <c r="J5" s="125"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="29" t="s">
         <v>160</v>
       </c>
@@ -13563,10 +13563,10 @@
       <c r="E6" s="40">
         <v>53.2</v>
       </c>
-      <c r="F6" s="142" t="s">
+      <c r="F6" s="134" t="s">
         <v>178</v>
       </c>
-      <c r="G6" s="143"/>
+      <c r="G6" s="135"/>
       <c r="H6" s="32">
         <v>4</v>
       </c>
@@ -13575,7 +13575,7 @@
       </c>
       <c r="J6" s="33"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="29" t="s">
         <v>161</v>
       </c>
@@ -13583,18 +13583,18 @@
         <v>180</v>
       </c>
       <c r="D7" s="45"/>
-      <c r="E7" s="144" t="s">
+      <c r="E7" s="136" t="s">
         <v>180</v>
       </c>
-      <c r="F7" s="145"/>
-      <c r="G7" s="143"/>
+      <c r="F7" s="137"/>
+      <c r="G7" s="135"/>
       <c r="H7" s="32">
         <v>4</v>
       </c>
       <c r="I7" s="41"/>
       <c r="J7" s="33"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B8" s="29" t="s">
         <v>162</v>
       </c>
@@ -13619,7 +13619,7 @@
       </c>
       <c r="J8" s="33"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B9" s="121" t="s">
         <v>197</v>
       </c>
@@ -13642,7 +13642,7 @@
       <c r="I9" s="41"/>
       <c r="J9" s="33"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="121" t="s">
         <v>196</v>
       </c>
@@ -13665,7 +13665,7 @@
       <c r="I10" s="41"/>
       <c r="J10" s="33"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="29" t="s">
         <v>163</v>
       </c>
@@ -13684,7 +13684,7 @@
       </c>
       <c r="J11" s="33"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="29" t="s">
         <v>164</v>
       </c>
@@ -13707,7 +13707,7 @@
       <c r="I12" s="41"/>
       <c r="J12" s="33"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="29" t="s">
         <v>165</v>
       </c>
@@ -13724,7 +13724,7 @@
       <c r="I13" s="41"/>
       <c r="J13" s="33"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" s="29" t="s">
         <v>184</v>
       </c>
@@ -13741,7 +13741,7 @@
       <c r="I14" s="41"/>
       <c r="J14" s="33"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" s="29" t="s">
         <v>185</v>
       </c>
@@ -13758,7 +13758,7 @@
       <c r="I15" s="41"/>
       <c r="J15" s="33"/>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="29" t="s">
         <v>186</v>
       </c>
@@ -13775,7 +13775,7 @@
       <c r="I16" s="41"/>
       <c r="J16" s="33"/>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="29" t="s">
         <v>166</v>
       </c>
@@ -13792,7 +13792,7 @@
       <c r="I17" s="41"/>
       <c r="J17" s="33"/>
     </row>
-    <row r="18" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="102" t="s">
         <v>182</v>
       </c>
@@ -13809,7 +13809,7 @@
       <c r="I18" s="124"/>
       <c r="J18" s="126"/>
     </row>
-    <row r="19" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="109" t="s">
         <v>187</v>
       </c>
@@ -13827,16 +13827,16 @@
       <c r="I19" s="115"/>
       <c r="J19" s="27"/>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B20" s="12"/>
       <c r="I20" s="116"/>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B21" s="117" t="s">
         <v>167</v>
       </c>
-      <c r="C21" s="142"/>
-      <c r="D21" s="146"/>
+      <c r="C21" s="134"/>
+      <c r="D21" s="138"/>
       <c r="E21" s="118" t="s">
         <v>122</v>
       </c>
@@ -13853,7 +13853,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" s="117" t="s">
         <v>168</v>
       </c>

</xml_diff>